<commit_message>
fix(course manager): fix course manager login
</commit_message>
<xml_diff>
--- a/doc/templates/Hango_Exam_Import_Template.xlsx
+++ b/doc/templates/Hango_Exam_Import_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Summer2026\SEP490\project\HanGo\doc\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFE8D0F-1B02-451C-A992-48618C837AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709105CE-D2B7-423C-AA89-485C0C458CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README_AND_RULES" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="69">
   <si>
     <t>2. Sheets to fill in:</t>
   </si>
@@ -36,9 +36,6 @@
     <t>4. After filling in the information, upload this file to the system.</t>
   </si>
   <si>
-    <t xml:space="preserve">   The system will automatically generate the entire course structure.</t>
-  </si>
-  <si>
     <t>Title</t>
   </si>
   <si>
@@ -51,12 +48,6 @@
     <t>Thumbnail URL</t>
   </si>
   <si>
-    <t>Simple Present</t>
-  </si>
-  <si>
-    <t>Simple Past</t>
-  </si>
-  <si>
     <t>Order Index</t>
   </si>
   <si>
@@ -99,12 +90,6 @@
     <t>EXAM OVERVIEW</t>
   </si>
   <si>
-    <t>EXAM_001</t>
-  </si>
-  <si>
-    <t>EXAM_002</t>
-  </si>
-  <si>
     <t xml:space="preserve">   - Exam: Main exam information</t>
   </si>
   <si>
@@ -123,12 +108,6 @@
     <t>Passing Score</t>
   </si>
   <si>
-    <t>This exam provides all knowledges about simple present tense</t>
-  </si>
-  <si>
-    <t>This exam provides all knowledges about simple past tense</t>
-  </si>
-  <si>
     <t xml:space="preserve">   - Question Count must be greater than 2 and less than or equal to 100</t>
   </si>
   <si>
@@ -249,25 +228,7 @@
     <t xml:space="preserve">   - Passage Text(optional): contains the content of the paragraph in the multiple question</t>
   </si>
   <si>
-    <t>tttt</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>abc</t>
-  </si>
-  <si>
-    <t>phonetics</t>
-  </si>
-  <si>
-    <t>easy</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
-    <t>medium</t>
+    <t xml:space="preserve">   The system will automatically generate the entire exam structure.</t>
   </si>
 </sst>
 </file>
@@ -503,25 +464,25 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -841,7 +802,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" ht="22.8">
       <c r="A1" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="22.8">
@@ -849,7 +810,7 @@
     </row>
     <row r="3" spans="1:3" ht="15.6">
       <c r="A3" s="10" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B3" s="11"/>
     </row>
@@ -865,13 +826,13 @@
     </row>
     <row r="6" spans="1:3" ht="15">
       <c r="A6" s="18" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B6" s="11"/>
     </row>
     <row r="7" spans="1:3" ht="15">
       <c r="A7" s="18" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B7" s="11"/>
     </row>
@@ -893,242 +854,242 @@
     </row>
     <row r="11" spans="1:3" customFormat="1">
       <c r="A11" s="19" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B11" s="14"/>
     </row>
     <row r="12" spans="1:3" customFormat="1">
       <c r="A12" s="19" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B12" s="14"/>
     </row>
     <row r="13" spans="1:3" customFormat="1">
       <c r="A13" s="19" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B13" s="14"/>
     </row>
     <row r="14" spans="1:3" customFormat="1" ht="14.4" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B14" s="19"/>
       <c r="C14" s="14"/>
     </row>
     <row r="15" spans="1:3" customFormat="1">
       <c r="A15" s="19" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B15" s="14"/>
     </row>
     <row r="16" spans="1:3" customFormat="1">
       <c r="A16" s="19" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B16" s="14"/>
     </row>
     <row r="17" spans="1:2" customFormat="1">
       <c r="A17" s="19" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B17" s="14"/>
     </row>
     <row r="18" spans="1:2" customFormat="1">
       <c r="A18" s="19" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B18" s="14"/>
     </row>
     <row r="19" spans="1:2" customFormat="1">
       <c r="A19" s="19" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B19" s="14"/>
     </row>
     <row r="20" spans="1:2" customFormat="1">
       <c r="A20" s="19" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B20" s="14"/>
     </row>
     <row r="21" spans="1:2" customFormat="1">
       <c r="A21" s="19" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B21" s="14"/>
     </row>
     <row r="22" spans="1:2" customFormat="1">
       <c r="A22" s="19" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B22" s="14"/>
     </row>
     <row r="23" spans="1:2" customFormat="1">
       <c r="A23" s="19" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B23" s="14"/>
     </row>
     <row r="24" spans="1:2" customFormat="1">
       <c r="A24" s="19" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B24" s="14"/>
     </row>
     <row r="25" spans="1:2" customFormat="1">
       <c r="A25" s="19" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B25" s="14"/>
     </row>
     <row r="26" spans="1:2" customFormat="1">
       <c r="A26" s="19" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B26" s="14"/>
     </row>
     <row r="27" spans="1:2" customFormat="1">
       <c r="A27" s="19" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B27" s="14"/>
     </row>
     <row r="28" spans="1:2" customFormat="1">
       <c r="A28" s="19" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B28" s="14"/>
     </row>
     <row r="29" spans="1:2" customFormat="1">
       <c r="A29" s="19" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B29" s="14"/>
     </row>
     <row r="30" spans="1:2" customFormat="1">
       <c r="A30" s="19" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B30" s="14"/>
     </row>
     <row r="31" spans="1:2" customFormat="1">
       <c r="A31" s="19" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B31" s="14"/>
     </row>
     <row r="32" spans="1:2" customFormat="1">
       <c r="A32" s="19" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B32" s="14"/>
     </row>
     <row r="33" spans="1:2" customFormat="1">
       <c r="A33" s="19" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B33" s="14"/>
     </row>
     <row r="34" spans="1:2" customFormat="1">
       <c r="A34" s="19" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B34" s="14"/>
     </row>
     <row r="35" spans="1:2" customFormat="1">
       <c r="A35" s="19" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B35" s="14"/>
     </row>
     <row r="36" spans="1:2" customFormat="1">
       <c r="A36" s="19" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B36" s="14"/>
     </row>
     <row r="37" spans="1:2" customFormat="1">
       <c r="A37" s="19" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B37" s="14"/>
     </row>
     <row r="38" spans="1:2" customFormat="1">
       <c r="A38" s="19" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B38" s="14"/>
     </row>
     <row r="39" spans="1:2" customFormat="1">
       <c r="A39" s="19" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B39" s="14"/>
     </row>
     <row r="40" spans="1:2" customFormat="1">
       <c r="A40" s="19" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B40" s="14"/>
     </row>
     <row r="41" spans="1:2" customFormat="1">
       <c r="A41" s="19" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B41" s="14"/>
     </row>
     <row r="42" spans="1:2" customFormat="1">
       <c r="A42" s="19" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B42" s="14"/>
     </row>
     <row r="43" spans="1:2" customFormat="1">
       <c r="A43" s="19" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B43" s="14"/>
     </row>
     <row r="44" spans="1:2" customFormat="1">
       <c r="A44" s="19" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B44" s="14"/>
     </row>
     <row r="45" spans="1:2" customFormat="1">
       <c r="A45" s="19" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B45" s="14"/>
     </row>
     <row r="46" spans="1:2" customFormat="1">
       <c r="A46" s="19" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B46" s="14"/>
     </row>
     <row r="47" spans="1:2" customFormat="1">
       <c r="A47" s="19" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B47" s="14"/>
     </row>
     <row r="48" spans="1:2" customFormat="1">
       <c r="A48" s="19" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B48" s="14"/>
     </row>
     <row r="49" spans="1:2" customFormat="1">
       <c r="A49" s="19" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B49" s="14"/>
     </row>
     <row r="50" spans="1:2" customFormat="1">
       <c r="A50" s="19" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B50" s="14"/>
     </row>
@@ -1140,7 +1101,7 @@
     </row>
     <row r="52" spans="1:2" customFormat="1">
       <c r="A52" s="13" t="s">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="B52" s="14"/>
     </row>
@@ -1206,227 +1167,198 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22.8">
-      <c r="A1" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="A1" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" ht="30" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
       <c r="D2" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" s="6"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="23">
-        <v>20</v>
-      </c>
-      <c r="E3" s="23">
-        <v>7</v>
-      </c>
-      <c r="F3" s="23"/>
+      <c r="A3" s="25"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+      <c r="A6" s="25"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="23">
-        <v>10</v>
-      </c>
-      <c r="E8" s="23">
-        <v>7</v>
-      </c>
-      <c r="F8" s="23"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="22"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="25"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="23"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="23"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="25"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="23"/>
     </row>
     <row r="16" spans="1:7" ht="12" customHeight="1">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="25"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="23"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="26"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="24"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="22"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="25"/>
+      <c r="A19" s="25"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="23"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="25"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="23"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="25"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="23"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="26"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="F18:F22"/>
-    <mergeCell ref="D3:D7"/>
-    <mergeCell ref="D8:D12"/>
-    <mergeCell ref="D13:D17"/>
-    <mergeCell ref="D18:D22"/>
-    <mergeCell ref="E3:E7"/>
-    <mergeCell ref="E8:E12"/>
-    <mergeCell ref="E13:E17"/>
-    <mergeCell ref="E18:E22"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A8:A12"/>
@@ -1443,6 +1375,15 @@
     <mergeCell ref="F3:F7"/>
     <mergeCell ref="F8:F12"/>
     <mergeCell ref="F13:F17"/>
+    <mergeCell ref="F18:F22"/>
+    <mergeCell ref="D3:D7"/>
+    <mergeCell ref="D8:D12"/>
+    <mergeCell ref="D13:D17"/>
+    <mergeCell ref="D18:D22"/>
+    <mergeCell ref="E3:E7"/>
+    <mergeCell ref="E8:E12"/>
+    <mergeCell ref="E13:E17"/>
+    <mergeCell ref="E18:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1465,134 +1406,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="22.8">
-      <c r="C1" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
+      <c r="C1" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="E2" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="G2" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="H2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="I2" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="J2" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="K2" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="20" t="s">
-        <v>21</v>
-      </c>
       <c r="L2" s="20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M2" s="20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="19.95" customHeight="1">
-      <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-      <c r="I3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" t="s">
-        <v>77</v>
-      </c>
-      <c r="K3" t="s">
-        <v>78</v>
-      </c>
-      <c r="L3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="19.95" customHeight="1">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-      <c r="I4" t="s">
-        <v>80</v>
-      </c>
-      <c r="J4" t="s">
-        <v>77</v>
-      </c>
-      <c r="K4" t="s">
-        <v>78</v>
-      </c>
-      <c r="L4" t="s">
-        <v>81</v>
-      </c>
-    </row>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="19.95" customHeight="1"/>
+    <row r="4" spans="1:13" ht="19.95" customHeight="1"/>
     <row r="5" spans="1:13" ht="19.95" customHeight="1"/>
     <row r="6" spans="1:13" ht="19.95" customHeight="1"/>
     <row r="7" spans="1:13" ht="19.95" customHeight="1"/>

</xml_diff>